<commit_message>
update example excel asset
</commit_message>
<xml_diff>
--- a/plan/pubgen/samples/BAB_01_2025.xlsx
+++ b/plan/pubgen/samples/BAB_01_2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\designcraft\plan\pubgen\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35ED9310-97B0-41D2-B543-16E99BA7DB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C000D459-01F6-4ED4-8D1C-55989C1A5B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9600" yWindow="4770" windowWidth="28800" windowHeight="9285" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="71">
   <si>
     <t>Warungbambu</t>
   </si>
@@ -278,6 +278,9 @@
   </si>
   <si>
     <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_pict2.png</t>
+  </si>
+  <si>
+    <t>Kata Pengantar</t>
   </si>
 </sst>
 </file>
@@ -943,30 +946,38 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7036A343-3A5A-488B-8DC0-22E63F44947D}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>66</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update sample files and templates
Refreshes the authored BAB_01 workbook and the three designcraft templates re-saved by the current build.
</commit_message>
<xml_diff>
--- a/plan/pubgen/samples/BAB_01_2025.xlsx
+++ b/plan/pubgen/samples/BAB_01_2025.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\designcraft-modular\plan\pubgen\samples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\designcraft\plan\pubgen\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55FDFE92-F0CE-43E6-8BD8-D088D276EE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81B7DC11-11D5-4737-AF2B-C83AEE9218A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6690" yWindow="6435" windowWidth="28800" windowHeight="9285" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COVER" sheetId="7" r:id="rId1"/>
@@ -29,6 +29,17 @@
     <definedName name="_Toc202275225" localSheetId="8">'01_01'!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -156,30 +167,6 @@
   </si>
   <si>
     <t>002</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\G00.rtf</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\G01.rtf</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\G02.rtf</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\images\city_skyline.jpg</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\images\city_landscape.jpg</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\images\bps_logo.png</t>
-  </si>
-  <si>
-    <t>F:\Github\designcraft\plan\pubgen\samples\A02.rtf</t>
-  </si>
-  <si>
-    <t>F:\Github\designcraft\plan\pubgen\samples\infografik_01.png</t>
   </si>
   <si>
     <t>Tabel 01.01 Luas Daerah Menurut Desa/Kelurahan di Kecamatan  Karawang Timur, 2025</t>
@@ -253,9 +240,6 @@
     <t>dividers/special_infographic_divider</t>
   </si>
   <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\R01.rtf</t>
-  </si>
-  <si>
     <t>KECAMATAN KARAWANG TIMUR</t>
   </si>
   <si>
@@ -265,22 +249,49 @@
     <t>Bab 01  Geografi</t>
   </si>
   <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01.rtf</t>
-  </si>
-  <si>
     <t>image2</t>
   </si>
   <si>
     <t>image1</t>
   </si>
   <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_pict1.jpg</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_pict2.png</t>
-  </si>
-  <si>
     <t>Kata Pengantar</t>
+  </si>
+  <si>
+    <t>E:\Github\designcraft\plan\pubgen\samples\G00.rtf</t>
+  </si>
+  <si>
+    <t>E:\Github\designcraft\plan\pubgen\samples\G01.rtf</t>
+  </si>
+  <si>
+    <t>E:\Github\designcraft\plan\pubgen\samples\G02.rtf</t>
+  </si>
+  <si>
+    <t>E:\Github\designcraft\plan\pubgen\samples\infografik_01.png</t>
+  </si>
+  <si>
+    <t>E:\Github\designcraft\plan\pubgen\samples\R01.rtf</t>
+  </si>
+  <si>
+    <t>E:\GitHub\designcraft\plan\pubgen\samples\B01_pict2.png</t>
+  </si>
+  <si>
+    <t>E:\GitHub\designcraft\plan\pubgen\samples\B01.rtf</t>
+  </si>
+  <si>
+    <t>E:\GitHub\designcraft\plan\pubgen\samples\B01_pict1.jpg</t>
+  </si>
+  <si>
+    <t>E:\Github\designcraft\plan\pubgen\samples\A02.rtf</t>
+  </si>
+  <si>
+    <t>E:\GitHub\designcraft\plan\pubgen\samples\images\city_skyline.jpg</t>
+  </si>
+  <si>
+    <t>E:\GitHub\designcraft\plan\pubgen\samples\images\city_landscape.jpg</t>
+  </si>
+  <si>
+    <t>E:\GitHub\designcraft\plan\pubgen\samples\images\bps_logo.png</t>
   </si>
 </sst>
 </file>
@@ -694,7 +705,7 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -702,7 +713,7 @@
         <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -750,7 +761,7 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -758,7 +769,7 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -766,7 +777,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -879,7 +890,7 @@
         <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +908,7 @@
         <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -910,18 +921,18 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -942,7 +953,7 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>41</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -960,7 +971,7 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -978,7 +989,7 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -996,7 +1007,7 @@
         <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -1004,7 +1015,7 @@
         <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1034,7 +1045,7 @@
         <v>8</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -1042,15 +1053,15 @@
         <v>9</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1070,19 +1081,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -1090,17 +1101,17 @@
     <row r="3" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A3" s="12"/>
       <c r="B3" s="9" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1151,7 +1162,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -1202,7 +1213,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B14" s="7">
         <f>SUM(B4:B13)</f>

</xml_diff>